<commit_message>
fix(inventory): match PEMFC alcohol to the source AE7 route
Mori et al. (2023), DOI 10.1016/j.ijhydene.2023.05.255, Table 1 specifies a seven-mol petrochemical ethoxylate, not AE>20. Select the existing RER petrochemical AE7 producer and product. Preserve the 4.58 g/kWe formula/cache, uncertainty and all other inputs. Document regional and chemical-class proxy limitations in the existing stack comment.

Scope: existing supplemental workbook inventories only. Approved as item 2 of ten on 2026-10-18.

Validation: exact edited-cell/ZIP-part scope, formula/cache round-trip and raw no-write ExcelImporter regression. Shared ecoinvent 3.8-3.12 checks are run after the batch; this does not constitute a full scenario rebuild.
</commit_message>
<xml_diff>
--- a/premise/data/additional_inventories/lci-fuel_cell.xlsx
+++ b/premise/data/additional_inventories/lci-fuel_cell.xlsx
@@ -1347,7 +1347,9 @@
       </c>
       <c r="B25" s="12" t="inlineStr">
         <is>
-          <t>LCI for a PEMFC fuel cell stack. Original size: 48 kWe, but normalized here to 1 kWe. Regarding geographical and time scope, production in Europe was considered based on current conditions. The reference year of the data is 2021 and data sets could be considered valid until 2024. The stack consists of 280 membrane electrode assembly (MEA) units with an active area of 200 cm2 each. The amount of Pt in the stack is 0.5425 g/kW, with a power density of 1.36 kW/kg. Operational time was set to 20,000 h at power of 1 kWe. Due to the degradation effects the hydrogen consumption must be increased to always generate the power of 1 kWe. In the case of dynamic operational regime 5 replacements (Nd = 5) of the PEMFC stack are included (lifetime of 3'800 hours per stack). Local PEMFC stack steel-identity correction, 2026-10-17 (approved). Mori et al. (2023), Life cycle sustainability assessment of a proton exchange membrane fuel cell technology for ecodesign purposes, DOI 10.1016/j.ijhydene.2023.05.255, Table 1, printed page 39676 (PDF page 4). https://repozitorij.uni-lj.si/Dokument.php?id=178494&amp;lang=slv The Steel product row reports 2.820 kg per 48 kWe stack, or 58.75 g/kWe, linked to DE: EAF Steel billet/Slab/Bloom Sphera. It is separate from the source stainless (450.47 g/kWe) and chromium-steel (17.75 g/kWe) entries. Replace only this 58.75 g input with steel production, electric, low-alloyed, Europe without Switzerland and Austria; product steel, low-alloyed. This ecoinvent European ordinary EAF-steel activity is a regional and grade proxy for the source German Sphera steel, not the identical source process or a documented exact alloy composition. Retain the original =58.75/1000 kg per 1 kWe stack formula, reference output, separate stainless inputs, steel-working service and other manufacturing coefficients. Inherited quantity uncertainty/pedigree fields are retained and do not quantify this supplier-proxy uncertainty. No added fabrication or yield factor, changed stack lifetime, or new primary/secondary trajectory. This mapping correction does not validate the complete stack, practical metal yields or suitability of the source 2021 light-vehicle design for other vehicles and future years.</t>
+          <t>APPROVED PEMFC ETHOXYLATED-ALCOHOL SOURCE MATCH, 2026-10-18. Mori et al. (2023), DOI 10.1016/j.ijhydene.2023.05.255, Table 1, printed page 39676 (https://repozitorij.uni-lj.si/Dokument.php?id=178494&amp;lang=slv), specifies C12-15 Alcohol (petro) Ethoxylate, 7 mol EO, 4.58 g/kWe. Replace AE&gt;20 with existing ethoxylated alcohol (AE7) production, petrochemical, RER. Retain =4.58/1000 kg/kWe, uncertainty and all other stack inputs. This European petrochemical supplier is a chemical-class and route proxy; exact chain-length distribution and measured supply are not established. No change to stack lifetime, platinum loading or any future reduction.
+PREVIOUS NOTES (retained as history; the correction above takes precedence):
+LCI for a PEMFC fuel cell stack. Original size: 48 kWe, but normalized here to 1 kWe. Regarding geographical and time scope, production in Europe was considered based on current conditions. The reference year of the data is 2021 and data sets could be considered valid until 2024. The stack consists of 280 membrane electrode assembly (MEA) units with an active area of 200 cm2 each. The amount of Pt in the stack is 0.5425 g/kW, with a power density of 1.36 kW/kg. Operational time was set to 20,000 h at power of 1 kWe. Due to the degradation effects the hydrogen consumption must be increased to always generate the power of 1 kWe. In the case of dynamic operational regime 5 replacements (Nd = 5) of the PEMFC stack are included (lifetime of 3'800 hours per stack). Local PEMFC stack steel-identity correction, 2026-10-17 (approved). Mori et al. (2023), Life cycle sustainability assessment of a proton exchange membrane fuel cell technology for ecodesign purposes, DOI 10.1016/j.ijhydene.2023.05.255, Table 1, printed page 39676 (PDF page 4). https://repozitorij.uni-lj.si/Dokument.php?id=178494&amp;lang=slv The Steel product row reports 2.820 kg per 48 kWe stack, or 58.75 g/kWe, linked to DE: EAF Steel billet/Slab/Bloom Sphera. It is separate from the source stainless (450.47 g/kWe) and chromium-steel (17.75 g/kWe) entries. Replace only this 58.75 g input with steel production, electric, low-alloyed, Europe without Switzerland and Austria; product steel, low-alloyed. This ecoinvent European ordinary EAF-steel activity is a regional and grade proxy for the source German Sphera steel, not the identical source process or a documented exact alloy composition. Retain the original =58.75/1000 kg per 1 kWe stack formula, reference output, separate stainless inputs, steel-working service and other manufacturing coefficients. Inherited quantity uncertainty/pedigree fields are retained and do not quantify this supplier-proxy uncertainty. No added fabrication or yield factor, changed stack lifetime, or new primary/secondary trajectory. This mapping correction does not validate the complete stack, practical metal yields or suitability of the source 2021 light-vehicle design for other vehicles and future years.</t>
         </is>
       </c>
       <c r="K25" s="13"/>
@@ -1925,15 +1927,19 @@
       </c>
     </row>
     <row r="37" spans="1:18" s="12" customFormat="1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A37" s="12" t="s">
-        <v>120</v>
+      <c r="A37" s="12" t="inlineStr">
+        <is>
+          <t>ethoxylated alcohol (AE7) production, petrochemical</t>
+        </is>
       </c>
       <c r="B37" s="12">
         <f>4.58/1000</f>
         <v>4.5799999999999999E-3</v>
       </c>
-      <c r="C37" s="12" t="s">
-        <v>16</v>
+      <c r="C37" s="12" t="inlineStr">
+        <is>
+          <t>RER</t>
+        </is>
       </c>
       <c r="D37" s="12" t="s">
         <v>13</v>
@@ -1941,8 +1947,10 @@
       <c r="F37" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="G37" s="12" t="s">
-        <v>121</v>
+      <c r="G37" s="12" t="inlineStr">
+        <is>
+          <t>ethoxylated alcohol (AE7)</t>
+        </is>
       </c>
       <c r="I37" s="12">
         <v>2</v>

</xml_diff>